<commit_message>
Compra de Componentes atrasados
Cambio de resistencia para CH224
</commit_message>
<xml_diff>
--- a/Componentes/ComponentesAtrasados.xlsx
+++ b/Componentes/ComponentesAtrasados.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Saile\Desktop\Github\ECG_Project\Componentes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4FD53018-7301-4B69-9DDB-71F238227B53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E402BF10-4843-487F-BB4D-2514EEA84EF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B89B2AA9-5016-4BB0-B292-57F2D3B7019D}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="116">
   <si>
     <t>Reference</t>
   </si>
@@ -83,9 +83,6 @@
     <t>D3</t>
   </si>
   <si>
-    <t>BAT54S</t>
-  </si>
-  <si>
     <t>D4</t>
   </si>
   <si>
@@ -125,9 +122,6 @@
     <t>J6</t>
   </si>
   <si>
-    <t>Conn_01x04_Pin</t>
-  </si>
-  <si>
     <t>R1,R2</t>
   </si>
   <si>
@@ -341,22 +335,40 @@
     <t>U5</t>
   </si>
   <si>
-    <t>Falta pero hay que revisar pertenencias</t>
-  </si>
-  <si>
     <t>Revisar en taller</t>
   </si>
   <si>
-    <t>Castana aliexpres</t>
-  </si>
-  <si>
-    <t>Aun no se cotiza</t>
-  </si>
-  <si>
     <t>Termica</t>
   </si>
   <si>
     <t>Tiene que ser de 1% de error</t>
+  </si>
+  <si>
+    <t>No se utilizará</t>
+  </si>
+  <si>
+    <t>****** 15 vs 27, faltarian 7 capacitores</t>
+  </si>
+  <si>
+    <t>Falta pero hay que revisar pertenencias, 30 vs 21 = deberian tener exacto</t>
+  </si>
+  <si>
+    <t>BAT54S / KL4</t>
+  </si>
+  <si>
+    <t>Pin Header 1.27mm</t>
+  </si>
+  <si>
+    <t>BAT1</t>
+  </si>
+  <si>
+    <t>Bateria LiPo</t>
+  </si>
+  <si>
+    <t>Se cambia por AMS1117</t>
+  </si>
+  <si>
+    <t>Hay que revisar pertenencias</t>
   </si>
 </sst>
 </file>
@@ -711,12 +723,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="5" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -831,6 +843,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -876,15 +925,44 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1260,22 +1338,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CBFE47C-7FDE-4C84-A66A-A45B69A0CBD5}">
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="40.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="70.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="26.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="40.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1288,826 +1367,875 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
+      <c r="F1" s="9"/>
+      <c r="H1" t="s">
         <v>0</v>
       </c>
-      <c r="H1" t="s">
-        <v>1</v>
-      </c>
       <c r="I1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" t="s">
         <v>2</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="4">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>6</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="H2" s="2">
+        <v>108</v>
+      </c>
+      <c r="F2" s="11"/>
+      <c r="H2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I2" s="2">
         <v>5</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="1">
         <v>6</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="15" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="1" t="s">
+      <c r="E3"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="1">
+      <c r="I3" s="1">
         <v>6</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="L3" s="7"/>
+    </row>
+    <row r="4" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="15" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="1" t="s">
+      <c r="E4"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="1">
+      <c r="I4" s="1">
         <v>2</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="G5" s="1" t="s">
+      <c r="L4" s="7"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="1">
-        <v>1</v>
-      </c>
-      <c r="I5" s="1" t="s">
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="15" t="s">
         <v>14</v>
       </c>
+      <c r="D5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="10"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="1">
+        <v>1</v>
+      </c>
       <c r="J5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="1">
-        <v>1</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="1" t="s">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="3">
+        <v>1</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F6" s="10"/>
+      <c r="H6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" s="1">
+        <v>1</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="1">
-        <v>1</v>
-      </c>
-      <c r="I6" s="1" t="s">
+      <c r="K6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J6" s="1" t="s">
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="4">
+        <v>1</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="F7" s="11"/>
+      <c r="H7" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="4">
-        <v>1</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="G7" s="1" t="s">
+      <c r="I7" s="1">
+        <v>1</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="4">
+        <v>1</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="F8" s="11"/>
+      <c r="H8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="1">
+        <v>2</v>
+      </c>
+      <c r="J8" s="1">
+        <v>510</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="4">
+        <v>1</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="F9" s="11"/>
+      <c r="H9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I9" s="1">
+        <v>2</v>
+      </c>
+      <c r="J9" s="1">
+        <v>51</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="F10" s="10"/>
+      <c r="H10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I10" s="1">
+        <v>3</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="1">
+        <v>1</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="10"/>
+      <c r="H11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I11" s="1">
+        <v>4</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" s="4">
+        <v>1</v>
+      </c>
+      <c r="C12" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="1">
-        <v>1</v>
-      </c>
-      <c r="I7" s="1" t="s">
+      <c r="D12" s="4"/>
+      <c r="F12" s="11"/>
+      <c r="H12" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="I12" s="2">
+        <v>1</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="4">
+        <v>2</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="F13" s="11"/>
+      <c r="H13" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I13" s="1">
+        <v>4</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="4">
+        <v>1</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="F14" s="11"/>
+      <c r="H14" s="2" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="5">
-        <v>1</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="G8" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="H8" s="1">
+      <c r="I14" s="2">
+        <v>7</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="1">
         <v>2</v>
       </c>
-      <c r="I8" s="1">
+      <c r="C15" s="15">
         <v>510</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="5">
-        <v>1</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" t="s">
-        <v>108</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H9" s="1">
+      <c r="D15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" s="10"/>
+      <c r="H15" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I15" s="1">
         <v>2</v>
       </c>
-      <c r="I9" s="1">
-        <v>51</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="5">
-        <v>1</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" s="5"/>
-      <c r="G10" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H10" s="1">
-        <v>3</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="1">
-        <v>1</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" s="1"/>
-      <c r="G11" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="H11" s="1">
-        <v>4</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="1">
-        <v>1</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="H12" s="2">
-        <v>1</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13" s="5">
-        <v>1</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="5"/>
-      <c r="G13" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="H13" s="1">
-        <v>4</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" s="5">
-        <v>2</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="5"/>
-      <c r="G14" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="H14" s="2">
-        <v>7</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="J14" s="2" t="s">
+      <c r="J15" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="5">
-        <v>1</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="5"/>
-      <c r="G15" s="1" t="s">
+      <c r="K15" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="H15" s="1">
-        <v>2</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B16" s="1">
         <v>2</v>
       </c>
-      <c r="C16" s="1">
-        <v>510</v>
+      <c r="C16" s="15">
+        <v>51</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="F16" s="10"/>
+      <c r="H16" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="I16" s="1">
+        <v>2</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="K16" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="H16" s="1">
-        <v>2</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B17" s="1">
+        <v>3</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F17" s="10"/>
+      <c r="H17" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="I17" s="1">
+        <v>1</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="1">
+        <v>4</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="10"/>
+      <c r="H18" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I18" s="1">
+        <v>1</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="3">
         <v>2</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C19" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F19" s="20"/>
+      <c r="H19" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="I19" s="1">
+        <v>1</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="1">
+        <v>4</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" s="10"/>
+      <c r="H20" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="I20" s="1">
+        <v>1</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B21" s="2">
+        <v>10</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="H17" s="1">
-        <v>1</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="J17" s="1" t="s">
+      <c r="E21" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F21" s="11"/>
+      <c r="H21" s="1" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="1">
-        <v>3</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="H18" s="1">
-        <v>1</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="1">
-        <v>4</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="H19" s="1">
-        <v>1</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B20" s="2">
+      <c r="I21" s="1">
+        <v>1</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="1">
         <v>2</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="H20" s="1">
-        <v>1</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B21" s="1">
-        <v>4</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="H21" s="1">
-        <v>1</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B22" s="2">
-        <v>10</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D22" s="2" t="s">
+      <c r="C22" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="E22" s="6" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D22" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F22" s="10"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B23" s="1">
         <v>2</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>55</v>
+      <c r="C23" s="15" t="s">
+        <v>56</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="1">
-        <v>2</v>
-      </c>
-      <c r="C24" s="1" t="s">
+      <c r="F23" s="10"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="B24" s="4">
+        <v>5</v>
+      </c>
+      <c r="C24" s="14" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
+      <c r="D24" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E24" s="7"/>
+      <c r="F24" s="11"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B25" s="5">
-        <v>5</v>
-      </c>
-      <c r="C25" s="5" t="s">
+      <c r="B25" s="4">
+        <v>1</v>
+      </c>
+      <c r="C25" s="14">
+        <v>120</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D25" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="5" t="s">
+      <c r="F25" s="11"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="5">
-        <v>1</v>
-      </c>
-      <c r="C26" s="5">
-        <v>120</v>
-      </c>
-      <c r="D26" s="5" t="s">
+      <c r="B26" s="4">
+        <v>1</v>
+      </c>
+      <c r="C26" s="14">
+        <v>470</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
+      <c r="F26" s="11"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B27" s="5">
-        <v>1</v>
-      </c>
-      <c r="C27" s="5">
-        <v>470</v>
-      </c>
-      <c r="D27" s="5" t="s">
+      <c r="B27" s="4">
+        <v>1</v>
+      </c>
+      <c r="C27" s="14">
+        <v>47</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="F27" s="11"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="5" t="s">
+      <c r="B28" s="4">
+        <v>1</v>
+      </c>
+      <c r="C28" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="B28" s="5">
-        <v>1</v>
-      </c>
-      <c r="C28" s="5">
-        <v>47</v>
-      </c>
-      <c r="D28" s="5"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
+      <c r="D28" s="4"/>
+      <c r="F28" s="11"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B29" s="5">
-        <v>1</v>
-      </c>
-      <c r="C29" s="5" t="s">
+      <c r="B29" s="3">
+        <v>1</v>
+      </c>
+      <c r="C29" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D29" s="5"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D29" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F29" s="11"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>69</v>
       </c>
       <c r="B30" s="4">
         <v>1</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="14">
+        <v>0.3</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F30" s="11"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="D30" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
+      <c r="B31" s="8">
+        <v>1</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F31" s="10"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B31" s="5">
-        <v>1</v>
-      </c>
-      <c r="C31" s="5">
-        <v>0.3</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="7" t="s">
+      <c r="B32" s="4">
+        <v>1</v>
+      </c>
+      <c r="C32" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="B32" s="7">
-        <v>1</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="E32" s="7" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="5" t="s">
+      <c r="D32" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F32" s="11"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B33" s="5">
-        <v>1</v>
-      </c>
-      <c r="C33" s="5" t="s">
+      <c r="B33" s="1">
+        <v>1</v>
+      </c>
+      <c r="C33" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="D33" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D33" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F33" s="10"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B34" s="1">
+        <v>1</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F34" s="10"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B35" s="1">
         <v>1</v>
       </c>
-      <c r="C35" s="1" t="s">
-        <v>76</v>
+      <c r="C35" s="15" t="s">
+        <v>79</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="B36" s="1">
-        <v>1</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="F35" s="10"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B36" s="4">
+        <v>1</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="F36" s="11"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B37" s="1">
-        <v>1</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>81</v>
+        <v>2</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>85</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B38" s="5">
-        <v>1</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B39" s="1">
+      <c r="F37" s="10"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B38" s="4">
+        <v>1</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="F38" s="11"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B39" s="4">
+        <v>1</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="D39" s="4"/>
+      <c r="F39" s="11"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B40" s="4">
+        <v>1</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="D40" s="4"/>
+      <c r="F40" s="11"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F41" s="10"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F42" s="20"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B43" s="4">
         <v>2</v>
       </c>
-      <c r="C39" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B40" s="5">
-        <v>1</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="B41" s="5">
-        <v>1</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="D41" s="5"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B42" s="5">
-        <v>1</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="D42" s="5"/>
+      <c r="C43" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D43" s="12">
+        <v>103450</v>
+      </c>
+      <c r="F43" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>